<commit_message>
Make schooling_start_age metadata-driven instead of hardcoded
Add optional `schooling_start_age` column to the `variables` sheet
(example template + instructions row), read in MAIN.R with a
fallback to 5 when blank, and pass it through to
add_loop_edu_ind_age_corrected() instead of the previous hardcoded
`schooling_start_age = 5`.
</commit_message>
<xml_diff>
--- a/input_tool/01_metadata/example_metadata_edu.xlsx
+++ b/input_tool/01_metadata/example_metadata_edu.xlsx
@@ -836,7 +836,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1574,22 +1574,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>strata_variables</t>
+          <t>variables</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>country_assessment</t>
+          <t>schooling_start_age</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Required</t>
-        </is>
-      </c>
-      <c r="D34" s="45" t="inlineStr">
-        <is>
-          <t>Must match the general/variables sheets.</t>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Age (in years) a child is expected to start school in this country. Used to correct implausible/miscoded ages before deriving school-cycle indicators. Leave blank to use the default of 5.</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>admin1 / admin2 / admin3</t>
+          <t>country_assessment</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="D35" s="45" t="inlineStr">
         <is>
-          <t>Column names for the three administrative levels used for disaggregation.</t>
+          <t>Must match the general/variables sheets.</t>
         </is>
       </c>
     </row>
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>stratum</t>
+          <t>admin1 / admin2 / admin3</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="D36" s="45" t="inlineStr">
         <is>
-          <t>Column name for the sampling stratum.</t>
+          <t>Column names for the three administrative levels used for disaggregation.</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>additional_stratum</t>
+          <t>stratum</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1655,7 +1655,7 @@
       </c>
       <c r="D37" s="45" t="inlineStr">
         <is>
-          <t>Column name for any additional stratification variable (e.g. population group).</t>
+          <t>Column name for the sampling stratum.</t>
         </is>
       </c>
     </row>
@@ -1667,39 +1667,57 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>additional_stratum</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Required</t>
+        </is>
+      </c>
+      <c r="D38" s="45" t="inlineStr">
+        <is>
+          <t>Column name for any additional stratification variable (e.g. population group).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>strata_variables</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>add_col1 ... add_col9</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
-      <c r="D38" s="45" t="inlineStr">
+      <c r="D39" s="45" t="inlineStr">
         <is>
           <t>Extra disaggregation/grouping columns specific to this country's analysis, as many as needed.</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr"/>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" s="45" t="inlineStr"/>
-    </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="D40" s="45" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>country code 00L</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" s="45" t="inlineStr">
+      <c r="D41" s="45" t="inlineStr">
         <is>
           <t>A fictional country ("Lemuria") kept in this file on purpose. It has several required fields intentionally left blank so you can set country_assessment &lt;- "00L" in MAIN.R and see exactly what the configuration-validation error message looks like, without touching real country data.</t>
         </is>
@@ -2064,7 +2082,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE21"/>
+  <dimension ref="A1:AF21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20.44140625" customWidth="1" min="1" max="1"/>
@@ -2237,6 +2255,11 @@
       <c r="AE1" s="14" t="inlineStr">
         <is>
           <t>cannot_do</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>schooling_start_age</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated version od the metadata file
</commit_message>
<xml_diff>
--- a/input_tool/01_metadata/example_metadata_edu.xlsx
+++ b/input_tool/01_metadata/example_metadata_edu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\EduAnalysisTool-v2-worktrees\main-config-validation\input_tool\01_metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlbertoRAMIREZ\Desktop\EduAnalysisTool DEMO\EduAnalysisTool-main\input_tool\01_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C83B4BE-A6DD-46E2-BE7B-A4C70AF62B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77648E68-B3C3-4F18-A96B-540352D62AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3330" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="266">
   <si>
     <t>country_assessment</t>
   </si>
@@ -365,9 +365,6 @@
     <t>Root column name for the education-barrier question.</t>
   </si>
   <si>
-    <t>Root column name for the occupation-related disruption question, if asked in this survey.</t>
-  </si>
-  <si>
     <t>Column name for the non-formal-education yes/no question, if asked.</t>
   </si>
   <si>
@@ -395,30 +392,9 @@
     <t>Must match the general/variables sheets.</t>
   </si>
   <si>
-    <t>admin1 / admin2 / admin3</t>
-  </si>
-  <si>
-    <t>Column names for the three administrative levels used for disaggregation.</t>
-  </si>
-  <si>
     <t>stratum</t>
   </si>
   <si>
-    <t>Column name for the sampling stratum.</t>
-  </si>
-  <si>
-    <t>additional_stratum</t>
-  </si>
-  <si>
-    <t>Column name for any additional stratification variable (e.g. population group).</t>
-  </si>
-  <si>
-    <t>add_col1 ... add_col9</t>
-  </si>
-  <si>
-    <t>Extra disaggregation/grouping columns specific to this country's analysis, as many as needed.</t>
-  </si>
-  <si>
     <t>Testing</t>
   </si>
   <si>
@@ -846,6 +822,18 @@
   </si>
   <si>
     <t>edu_nonformal</t>
+  </si>
+  <si>
+    <t>Root column name for the school-occupation disruption question — school occupied by armed forces/non-state armed groups. Passed as humind's `attack` argument in add_loop_edu_disrupted_d() (an attacks-on-education category), then renamed to edu_disrupted_occupation_d.</t>
+  </si>
+  <si>
+    <t>First disaggregation level (e.g. admin1 or your primary reporting stratum) column name.</t>
+  </si>
+  <si>
+    <t>strata_lvl_2 ... strata_lvl_15</t>
+  </si>
+  <si>
+    <t>Additional disaggregation levels, as many as needed (admin2/3, sampling stratum, population group, or any other grouping variable), in any order — fill only as many as your analysis needs.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" style="16" customWidth="1"/>
@@ -1416,18 +1404,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
-        <v>71</v>
+        <v>119</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>73</v>
+        <v>120</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1435,13 +1420,13 @@
         <v>71</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1449,13 +1434,13 @@
         <v>71</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1463,13 +1448,13 @@
         <v>71</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1477,13 +1462,13 @@
         <v>71</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1491,13 +1476,13 @@
         <v>71</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1505,13 +1490,13 @@
         <v>71</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1519,27 +1504,27 @@
         <v>71</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1547,13 +1532,13 @@
         <v>71</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>154</v>
+        <v>88</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>210</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1561,27 +1546,27 @@
         <v>71</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>261</v>
+        <v>146</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1589,27 +1574,27 @@
         <v>71</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1617,13 +1602,13 @@
         <v>91</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>92</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1631,13 +1616,13 @@
         <v>91</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1645,13 +1630,13 @@
         <v>91</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1659,13 +1644,13 @@
         <v>91</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1673,13 +1658,13 @@
         <v>91</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1687,13 +1672,13 @@
         <v>91</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1701,13 +1686,13 @@
         <v>91</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1715,13 +1700,13 @@
         <v>91</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1729,13 +1714,13 @@
         <v>91</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1743,13 +1728,13 @@
         <v>91</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1757,13 +1742,13 @@
         <v>91</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1771,13 +1756,13 @@
         <v>91</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1785,13 +1770,13 @@
         <v>91</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1799,13 +1784,13 @@
         <v>91</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1813,13 +1798,13 @@
         <v>91</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1827,27 +1812,27 @@
         <v>91</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>108</v>
+        <v>262</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -1855,13 +1840,13 @@
         <v>91</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1869,13 +1854,13 @@
         <v>91</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1883,41 +1868,41 @@
         <v>91</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D35" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="17" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D36" s="16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1925,13 +1910,13 @@
         <v>91</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>31</v>
+        <v>113</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1939,94 +1924,69 @@
         <v>91</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>259</v>
+        <v>31</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="16" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>0</v>
+        <v>251</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>118</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>121</v>
+        <v>234</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>123</v>
+        <v>264</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D43" s="16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="B44" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="C44" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="16" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="B46" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D46" s="16" t="s">
-        <v>129</v>
+      <c r="D43" s="17" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2074,16 +2034,16 @@
         <v>88</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -2091,34 +2051,34 @@
         <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -2127,35 +2087,35 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -2178,22 +2138,22 @@
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -2204,22 +2164,22 @@
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -2352,30 +2312,30 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -2574,10 +2534,10 @@
         <v>31</v>
       </c>
       <c r="AG1" s="13" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="AH1" s="13" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -2637,28 +2597,28 @@
         <v>43</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>21</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="AB2" s="5" t="s">
         <v>27</v>
@@ -2667,10 +2627,10 @@
         <v>28</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="AE2" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="AF2" s="10">
         <v>5</v>
@@ -2714,7 +2674,7 @@
         <v>35</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -2740,7 +2700,7 @@
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="5" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
@@ -2779,47 +2739,47 @@
         <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="Q4" s="5"/>
       <c r="R4" s="5" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="U4" s="5"/>
       <c r="V4" s="5"/>
@@ -3023,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>36</v>
@@ -3050,7 +3010,7 @@
         <v>42</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="T7" s="5" t="s">
         <v>50</v>
@@ -3122,7 +3082,7 @@
         <v>41</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R8" s="5" t="s">
         <v>42</v>
@@ -3202,7 +3162,7 @@
         <v>41</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R9" s="5" t="s">
         <v>42</v>
@@ -3237,10 +3197,10 @@
         <v>54</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>34</v>
@@ -3291,10 +3251,10 @@
         <v>43</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
@@ -3365,7 +3325,7 @@
         <v>46</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="S11" s="5" t="s">
         <v>43</v>
@@ -3405,19 +3365,19 @@
         <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>36</v>
@@ -3438,7 +3398,7 @@
         <v>41</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R12" s="5" t="s">
         <v>42</v>
@@ -3473,13 +3433,13 @@
         <v>56</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E13" s="3">
         <v>10</v>
@@ -3497,7 +3457,7 @@
         <v>8</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>10</v>
@@ -3533,22 +3493,22 @@
         <v>50</v>
       </c>
       <c r="V13" s="5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="X13" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="Y13" s="5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="Z13" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="AA13" s="5" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="AB13" s="5" t="s">
         <v>27</v>
@@ -3557,10 +3517,10 @@
         <v>28</v>
       </c>
       <c r="AD13" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="AE13" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="AF13" s="5"/>
       <c r="AG13" s="5"/>
@@ -3579,25 +3539,25 @@
         <v>33</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E14" s="3">
         <v>8</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>36</v>
@@ -3690,7 +3650,7 @@
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>33</v>
@@ -3720,22 +3680,22 @@
         <v>35</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="M16" s="5" t="s">
         <v>38</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="P16" s="5" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="Q16" s="5"/>
       <c r="R16" s="5" t="s">
@@ -3770,7 +3730,7 @@
         <v>33</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>34</v>
@@ -3779,40 +3739,40 @@
         <v>9</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="R17" s="5"/>
       <c r="S17" s="5" t="s">
@@ -3841,7 +3801,7 @@
         <v>59</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>48</v>
@@ -3920,52 +3880,52 @@
         <v>33</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="P19" s="5" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="R19" s="5" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="S19" s="5" t="s">
         <v>43</v>
@@ -3999,7 +3959,7 @@
         <v>33</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="E20" s="3">
         <v>9</v>
@@ -4026,7 +3986,7 @@
         <v>37</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>39</v>
@@ -4041,16 +4001,16 @@
         <v>46</v>
       </c>
       <c r="R20" s="5" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="T20" s="5" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="V20" s="5"/>
       <c r="W20" s="5"/>
@@ -4131,10 +4091,10 @@
         <v>6</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>35</v>
@@ -4146,17 +4106,17 @@
         <v>11</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
       <c r="P22" s="5"/>
       <c r="Q22" s="5"/>
       <c r="R22" s="5" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
@@ -4225,49 +4185,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="J1" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="K1" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="M1" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="N1" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="O1" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="P1" s="14" t="s">
         <v>248</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="J1" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="K1" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="N1" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="O1" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="P1" s="14" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
@@ -4275,19 +4235,19 @@
         <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -4305,16 +4265,16 @@
         <v>32</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -4352,22 +4312,22 @@
         <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -4384,31 +4344,31 @@
         <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -4599,22 +4559,22 @@
     </row>
     <row r="16" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>

</xml_diff>

<commit_message>
Update of supporting files
</commit_message>
<xml_diff>
--- a/input_tool/01_metadata/example_metadata_edu.xlsx
+++ b/input_tool/01_metadata/example_metadata_edu.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\albertoramirez\Projects\EduAnalysisTool-v2-worktrees\main-config-validation\input_tool\01_metadata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlbertoRAMIREZ\Desktop\EduAnalysisTool DEMO\EduAnalysisTool-main\input_tool\01_metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C83B4BE-A6DD-46E2-BE7B-A4C70AF62B84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77648E68-B3C3-4F18-A96B-540352D62AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-3330" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="instructions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="719" uniqueCount="266">
   <si>
     <t>country_assessment</t>
   </si>
@@ -365,9 +365,6 @@
     <t>Root column name for the education-barrier question.</t>
   </si>
   <si>
-    <t>Root column name for the occupation-related disruption question, if asked in this survey.</t>
-  </si>
-  <si>
     <t>Column name for the non-formal-education yes/no question, if asked.</t>
   </si>
   <si>
@@ -395,30 +392,9 @@
     <t>Must match the general/variables sheets.</t>
   </si>
   <si>
-    <t>admin1 / admin2 / admin3</t>
-  </si>
-  <si>
-    <t>Column names for the three administrative levels used for disaggregation.</t>
-  </si>
-  <si>
     <t>stratum</t>
   </si>
   <si>
-    <t>Column name for the sampling stratum.</t>
-  </si>
-  <si>
-    <t>additional_stratum</t>
-  </si>
-  <si>
-    <t>Column name for any additional stratification variable (e.g. population group).</t>
-  </si>
-  <si>
-    <t>add_col1 ... add_col9</t>
-  </si>
-  <si>
-    <t>Extra disaggregation/grouping columns specific to this country's analysis, as many as needed.</t>
-  </si>
-  <si>
     <t>Testing</t>
   </si>
   <si>
@@ -846,6 +822,18 @@
   </si>
   <si>
     <t>edu_nonformal</t>
+  </si>
+  <si>
+    <t>Root column name for the school-occupation disruption question — school occupied by armed forces/non-state armed groups. Passed as humind's `attack` argument in add_loop_edu_disrupted_d() (an attacks-on-education category), then renamed to edu_disrupted_occupation_d.</t>
+  </si>
+  <si>
+    <t>First disaggregation level (e.g. admin1 or your primary reporting stratum) column name.</t>
+  </si>
+  <si>
+    <t>strata_lvl_2 ... strata_lvl_15</t>
+  </si>
+  <si>
+    <t>Additional disaggregation levels, as many as needed (admin2/3, sampling stratum, population group, or any other grouping variable), in any order — fill only as many as your analysis needs.</t>
   </si>
 </sst>
 </file>
@@ -1392,7 +1380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16" style="16" customWidth="1"/>
@@ -1416,18 +1404,15 @@
         <v>70</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="16" t="s">
-        <v>71</v>
+        <v>119</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>73</v>
+        <v>120</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1435,13 +1420,13 @@
         <v>71</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1449,13 +1434,13 @@
         <v>71</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C4" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1463,13 +1448,13 @@
         <v>71</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C5" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1477,13 +1462,13 @@
         <v>71</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C6" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1491,13 +1476,13 @@
         <v>71</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C7" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1505,13 +1490,13 @@
         <v>71</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C8" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1519,27 +1504,27 @@
         <v>71</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C9" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1547,13 +1532,13 @@
         <v>71</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>154</v>
+        <v>88</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>210</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1561,27 +1546,27 @@
         <v>71</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>261</v>
+        <v>146</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="16" t="s">
         <v>71</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1589,27 +1574,27 @@
         <v>71</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="C14" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="16" t="s">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>0</v>
+        <v>254</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1617,13 +1602,13 @@
         <v>91</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C16" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>92</v>
+        <v>260</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1631,13 +1616,13 @@
         <v>91</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C17" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1645,13 +1630,13 @@
         <v>91</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C18" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1659,13 +1644,13 @@
         <v>91</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1673,13 +1658,13 @@
         <v>91</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C20" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1687,13 +1672,13 @@
         <v>91</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C21" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1701,13 +1686,13 @@
         <v>91</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C22" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1715,13 +1700,13 @@
         <v>91</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C23" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1729,13 +1714,13 @@
         <v>91</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C24" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1743,13 +1728,13 @@
         <v>91</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C25" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1757,13 +1742,13 @@
         <v>91</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C26" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1771,13 +1756,13 @@
         <v>91</v>
       </c>
       <c r="B27" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C27" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1785,13 +1770,13 @@
         <v>91</v>
       </c>
       <c r="B28" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C28" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1799,13 +1784,13 @@
         <v>91</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1813,13 +1798,13 @@
         <v>91</v>
       </c>
       <c r="B30" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C30" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1827,27 +1812,27 @@
         <v>91</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C31" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C32" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>108</v>
+        <v>262</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -1855,13 +1840,13 @@
         <v>91</v>
       </c>
       <c r="B33" s="16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1869,13 +1854,13 @@
         <v>91</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C34" s="16" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1883,41 +1868,41 @@
         <v>91</v>
       </c>
       <c r="B35" s="16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C35" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D35" s="16" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="D35" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="C36" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D36" s="17" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D36" s="16" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A37" s="16" t="s">
         <v>91</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C37" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1925,13 +1910,13 @@
         <v>91</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>31</v>
+        <v>113</v>
       </c>
       <c r="C38" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
@@ -1939,94 +1924,69 @@
         <v>91</v>
       </c>
       <c r="B39" s="16" t="s">
-        <v>259</v>
+        <v>31</v>
       </c>
       <c r="C39" s="16" t="s">
         <v>89</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A40" s="16" t="s">
-        <v>117</v>
+        <v>91</v>
       </c>
       <c r="B40" s="16" t="s">
-        <v>0</v>
+        <v>251</v>
       </c>
       <c r="C40" s="16" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>118</v>
+        <v>259</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B41" s="16" t="s">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="C41" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D41" s="17" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>121</v>
+        <v>234</v>
       </c>
       <c r="C42" s="16" t="s">
         <v>72</v>
       </c>
       <c r="D42" s="17" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A43" s="16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B43" s="16" t="s">
-        <v>123</v>
+        <v>264</v>
       </c>
       <c r="C43" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="D43" s="16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A44" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="B44" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="C44" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="D44" s="16" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="B46" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D46" s="16" t="s">
-        <v>129</v>
+      <c r="D43" s="17" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -2074,16 +2034,16 @@
         <v>88</v>
       </c>
       <c r="J1" s="9" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="K1" s="9" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>263</v>
+        <v>255</v>
       </c>
       <c r="M1" s="9" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -2091,34 +2051,34 @@
         <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
@@ -2127,35 +2087,35 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
@@ -2178,22 +2138,22 @@
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -2204,22 +2164,22 @@
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -2352,30 +2312,30 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -2574,10 +2534,10 @@
         <v>31</v>
       </c>
       <c r="AG1" s="13" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="AH1" s="13" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
     </row>
     <row r="2" spans="1:34" ht="15" thickTop="1" x14ac:dyDescent="0.3">
@@ -2637,28 +2597,28 @@
         <v>43</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="V2" s="10" t="s">
         <v>21</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="X2" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="Y2" s="5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="Z2" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="AA2" s="5" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="AB2" s="5" t="s">
         <v>27</v>
@@ -2667,10 +2627,10 @@
         <v>28</v>
       </c>
       <c r="AD2" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="AE2" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="AF2" s="10">
         <v>5</v>
@@ -2714,7 +2674,7 @@
         <v>35</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="L3" s="5" t="s">
         <v>37</v>
@@ -2740,7 +2700,7 @@
       </c>
       <c r="T3" s="5"/>
       <c r="U3" s="5" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
@@ -2779,47 +2739,47 @@
         <v>10</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="M4" s="5" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="O4" s="5" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="Q4" s="5"/>
       <c r="R4" s="5" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="S4" s="5" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="U4" s="5"/>
       <c r="V4" s="5"/>
@@ -3023,7 +2983,7 @@
         <v>8</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>36</v>
@@ -3050,7 +3010,7 @@
         <v>42</v>
       </c>
       <c r="S7" s="5" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="T7" s="5" t="s">
         <v>50</v>
@@ -3122,7 +3082,7 @@
         <v>41</v>
       </c>
       <c r="Q8" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R8" s="5" t="s">
         <v>42</v>
@@ -3202,7 +3162,7 @@
         <v>41</v>
       </c>
       <c r="Q9" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R9" s="5" t="s">
         <v>42</v>
@@ -3237,10 +3197,10 @@
         <v>54</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>34</v>
@@ -3291,10 +3251,10 @@
         <v>43</v>
       </c>
       <c r="T10" s="5" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="U10" s="5" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="V10" s="5"/>
       <c r="W10" s="5"/>
@@ -3365,7 +3325,7 @@
         <v>46</v>
       </c>
       <c r="R11" s="5" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="S11" s="5" t="s">
         <v>43</v>
@@ -3405,19 +3365,19 @@
         <v>11</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>36</v>
@@ -3438,7 +3398,7 @@
         <v>41</v>
       </c>
       <c r="Q12" s="5" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R12" s="5" t="s">
         <v>42</v>
@@ -3473,13 +3433,13 @@
         <v>56</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="E13" s="3">
         <v>10</v>
@@ -3497,7 +3457,7 @@
         <v>8</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>10</v>
@@ -3533,22 +3493,22 @@
         <v>50</v>
       </c>
       <c r="V13" s="5" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="W13" s="5" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="X13" s="5" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="Y13" s="5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="Z13" s="5" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="AA13" s="5" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="AB13" s="5" t="s">
         <v>27</v>
@@ -3557,10 +3517,10 @@
         <v>28</v>
       </c>
       <c r="AD13" s="5" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="AE13" s="5" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="AF13" s="5"/>
       <c r="AG13" s="5"/>
@@ -3579,25 +3539,25 @@
         <v>33</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="E14" s="3">
         <v>8</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>36</v>
@@ -3690,7 +3650,7 @@
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>33</v>
@@ -3720,22 +3680,22 @@
         <v>35</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="M16" s="5" t="s">
         <v>38</v>
       </c>
       <c r="N16" s="5" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="O16" s="5" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="P16" s="5" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="Q16" s="5"/>
       <c r="R16" s="5" t="s">
@@ -3770,7 +3730,7 @@
         <v>33</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>34</v>
@@ -3779,40 +3739,40 @@
         <v>9</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="O17" s="5" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="Q17" s="5" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="R17" s="5"/>
       <c r="S17" s="5" t="s">
@@ -3841,7 +3801,7 @@
         <v>59</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>48</v>
@@ -3920,52 +3880,52 @@
         <v>33</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="N19" s="5" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="O19" s="5" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="P19" s="5" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="Q19" s="5" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="R19" s="5" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="S19" s="5" t="s">
         <v>43</v>
@@ -3999,7 +3959,7 @@
         <v>33</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="E20" s="3">
         <v>9</v>
@@ -4026,7 +3986,7 @@
         <v>37</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="N20" s="5" t="s">
         <v>39</v>
@@ -4041,16 +4001,16 @@
         <v>46</v>
       </c>
       <c r="R20" s="5" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="S20" s="5" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="T20" s="5" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="U20" s="5" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="V20" s="5"/>
       <c r="W20" s="5"/>
@@ -4131,10 +4091,10 @@
         <v>6</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>35</v>
@@ -4146,17 +4106,17 @@
         <v>11</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="N22" s="5"/>
       <c r="O22" s="5"/>
       <c r="P22" s="5"/>
       <c r="Q22" s="5"/>
       <c r="R22" s="5" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="S22" s="5" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
@@ -4225,49 +4185,49 @@
         <v>0</v>
       </c>
       <c r="B1" s="14" t="s">
+        <v>234</v>
+      </c>
+      <c r="C1" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="D1" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="F1" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="G1" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="H1" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="J1" s="14" t="s">
         <v>242</v>
       </c>
-      <c r="C1" s="14" t="s">
+      <c r="K1" s="14" t="s">
         <v>243</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="L1" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="M1" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="N1" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="G1" s="14" t="s">
+      <c r="O1" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="H1" s="14" t="s">
+      <c r="P1" s="14" t="s">
         <v>248</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="J1" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="K1" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="L1" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="M1" s="14" t="s">
-        <v>253</v>
-      </c>
-      <c r="N1" s="14" t="s">
-        <v>254</v>
-      </c>
-      <c r="O1" s="14" t="s">
-        <v>255</v>
-      </c>
-      <c r="P1" s="14" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
@@ -4275,19 +4235,19 @@
         <v>66</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -4305,16 +4265,16 @@
         <v>32</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -4352,22 +4312,22 @@
         <v>45</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
@@ -4384,31 +4344,31 @@
         <v>47</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>145</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2"/>
@@ -4599,22 +4559,22 @@
     </row>
     <row r="16" spans="1:16" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>

</xml_diff>